<commit_message>
Add IDP Attitudes Survey 2026 (DOC-169) and correct 2025 results
- New idp-survey-2026.html: all 31 questions plus demographics as tables,
  with corrected 2025 figures and a comparable subsample column (n=725);
  fieldwork credited to Operativna Sotsiolohiya
- data/idp-survey/: results XLSX (about, results, verbatim other answers,
  corrections), long-format CSV and JSON
- Reissue data/tot_idp_polling.xlsx: Q8 had repeated the Q9 distribution;
  Q7 hard-to-say/refusal transposed; four 0.1pt rounding slips; added
  corrections sheet. Correction notice on idp-survey.html
- Dashboard Q11 bars: rounding fixes
- data.html card, catalogue entry, sitemap list, documents.js v=9

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/tot_idp_polling.xlsx
+++ b/data/tot_idp_polling.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Одномірки" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Інше(11)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Інше(12)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Виправлення (Corrections)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,8 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,13 +30,28 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F0EC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -48,8 +66,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z381"/>
+  <dimension ref="A1:F181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -425,7 +450,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
@@ -497,7 +521,7 @@
           <t>Населений пункт в якому я проживав до повномасштабного вторгнення був окупований, а зараз вже деокупований</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="1" t="n">
         <v>0.1248751248751249</v>
       </c>
     </row>
@@ -507,7 +531,7 @@
           <t>Населений пункт в якому я проживав до повномасштабного вторгнення був окупований, і зараз залишається окупованим</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="1" t="n">
         <v>0.8751248751248751</v>
       </c>
     </row>
@@ -526,7 +550,7 @@
           <t>Точно ні</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="1" t="n">
         <v>0.09290709290709291</v>
       </c>
     </row>
@@ -536,7 +560,7 @@
           <t>Скоріше ні</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="1" t="n">
         <v>0.02897102897102897</v>
       </c>
     </row>
@@ -546,7 +570,7 @@
           <t>Скоріше так</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" s="1" t="n">
         <v>0.06993006993006994</v>
       </c>
     </row>
@@ -556,7 +580,7 @@
           <t>Точно так</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="1" t="n">
         <v>0.8041958041958042</v>
       </c>
     </row>
@@ -566,7 +590,7 @@
           <t>Важко відповісти</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" s="1" t="n">
         <v>0.003996003996003996</v>
       </c>
     </row>
@@ -576,7 +600,7 @@
           <t>Не хочу відповідати</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -595,7 +619,7 @@
           <t>Повністю не ефективно</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="1" t="n">
         <v>0.4265734265734266</v>
       </c>
     </row>
@@ -605,7 +629,7 @@
           <t>Скоріше не ефективно</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" s="1" t="n">
         <v>0.3366633366633366</v>
       </c>
     </row>
@@ -615,7 +639,7 @@
           <t>Скоріше ефективно</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" s="1" t="n">
         <v>0.1478521478521478</v>
       </c>
     </row>
@@ -625,7 +649,7 @@
           <t>Повністю ефективно</t>
         </is>
       </c>
-      <c r="C26" t="n">
+      <c r="C26" s="1" t="n">
         <v>0.04895104895104895</v>
       </c>
     </row>
@@ -635,7 +659,7 @@
           <t>Важко відповісти</t>
         </is>
       </c>
-      <c r="C27" t="n">
+      <c r="C27" s="1" t="n">
         <v>0.03996003996003996</v>
       </c>
     </row>
@@ -645,7 +669,7 @@
           <t>Не хочу відповідати</t>
         </is>
       </c>
-      <c r="C28" t="n">
+      <c r="C28" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -664,7 +688,7 @@
           <t>Повністю не ефективно</t>
         </is>
       </c>
-      <c r="C32" t="n">
+      <c r="C32" s="1" t="n">
         <v>0.1728271728271728</v>
       </c>
     </row>
@@ -674,7 +698,7 @@
           <t>Скоріше не ефективно</t>
         </is>
       </c>
-      <c r="C33" t="n">
+      <c r="C33" s="1" t="n">
         <v>0.3156843156843157</v>
       </c>
     </row>
@@ -684,7 +708,7 @@
           <t>Скоріше ефективно</t>
         </is>
       </c>
-      <c r="C34" t="n">
+      <c r="C34" s="1" t="n">
         <v>0.3376623376623377</v>
       </c>
     </row>
@@ -694,7 +718,7 @@
           <t>Повністю ефективно</t>
         </is>
       </c>
-      <c r="C35" t="n">
+      <c r="C35" s="1" t="n">
         <v>0.07292707292707293</v>
       </c>
     </row>
@@ -704,7 +728,7 @@
           <t>Важко відповісти</t>
         </is>
       </c>
-      <c r="C36" t="n">
+      <c r="C36" s="1" t="n">
         <v>0.0999000999000999</v>
       </c>
     </row>
@@ -714,7 +738,7 @@
           <t>Не хочу відповідати</t>
         </is>
       </c>
-      <c r="C37" t="n">
+      <c r="C37" s="1" t="n">
         <v>0.000999000999000999</v>
       </c>
     </row>
@@ -733,7 +757,7 @@
           <t>Точно ні</t>
         </is>
       </c>
-      <c r="C41" t="n">
+      <c r="C41" s="1" t="n">
         <v>0.3756243756243756</v>
       </c>
     </row>
@@ -743,7 +767,7 @@
           <t>Скоріше ні</t>
         </is>
       </c>
-      <c r="C42" t="n">
+      <c r="C42" s="1" t="n">
         <v>0.1258741258741259</v>
       </c>
     </row>
@@ -753,7 +777,7 @@
           <t>Скоріше так</t>
         </is>
       </c>
-      <c r="C43" t="n">
+      <c r="C43" s="1" t="n">
         <v>0.1518481518481518</v>
       </c>
     </row>
@@ -763,7 +787,7 @@
           <t>Точно так</t>
         </is>
       </c>
-      <c r="C44" t="n">
+      <c r="C44" s="1" t="n">
         <v>0.3336663336663337</v>
       </c>
     </row>
@@ -773,8 +797,8 @@
           <t>Важко відповісти</t>
         </is>
       </c>
-      <c r="C45" t="n">
-        <v>0.005</v>
+      <c r="C45" s="1" t="n">
+        <v>0.007992007992007992</v>
       </c>
     </row>
     <row r="46">
@@ -783,8 +807,8 @@
           <t>Не хочу відповідати</t>
         </is>
       </c>
-      <c r="C46" t="n">
-        <v>0.008</v>
+      <c r="C46" s="1" t="n">
+        <v>0.004995004995004995</v>
       </c>
     </row>
     <row r="47"/>
@@ -802,8 +826,8 @@
           <t>Точно ні</t>
         </is>
       </c>
-      <c r="C50" t="n">
-        <v>0.03607214428857716</v>
+      <c r="C50" s="1" t="n">
+        <v>0.2615230460921844</v>
       </c>
     </row>
     <row r="51">
@@ -812,8 +836,8 @@
           <t>Скоріше ні</t>
         </is>
       </c>
-      <c r="C51" t="n">
-        <v>0.1432865731462926</v>
+      <c r="C51" s="1" t="n">
+        <v>0.3236472945891783</v>
       </c>
     </row>
     <row r="52">
@@ -822,8 +846,8 @@
           <t>Скоріше так</t>
         </is>
       </c>
-      <c r="C52" t="n">
-        <v>0.3647294589178356</v>
+      <c r="C52" s="1" t="n">
+        <v>0.1983967935871744</v>
       </c>
     </row>
     <row r="53">
@@ -832,8 +856,8 @@
           <t>Точно так</t>
         </is>
       </c>
-      <c r="C53" t="n">
-        <v>0.250501002004008</v>
+      <c r="C53" s="1" t="n">
+        <v>0.07615230460921844</v>
       </c>
     </row>
     <row r="54">
@@ -842,7 +866,7 @@
           <t>Важко відповісти</t>
         </is>
       </c>
-      <c r="C54" t="n">
+      <c r="C54" s="1" t="n">
         <v>0.1382765531062124</v>
       </c>
     </row>
@@ -852,7 +876,7 @@
           <t>Не хочу відповідати</t>
         </is>
       </c>
-      <c r="C55" t="n">
+      <c r="C55" s="1" t="n">
         <v>0.002</v>
       </c>
     </row>
@@ -871,7 +895,7 @@
           <t>Точно ні</t>
         </is>
       </c>
-      <c r="C59" t="n">
+      <c r="C59" s="1" t="n">
         <v>0.03607214428857716</v>
       </c>
     </row>
@@ -881,7 +905,7 @@
           <t>Скоріше ні</t>
         </is>
       </c>
-      <c r="C60" t="n">
+      <c r="C60" s="1" t="n">
         <v>0.1432865731462926</v>
       </c>
     </row>
@@ -891,7 +915,7 @@
           <t>Скоріше так</t>
         </is>
       </c>
-      <c r="C61" t="n">
+      <c r="C61" s="1" t="n">
         <v>0.3647294589178356</v>
       </c>
     </row>
@@ -901,7 +925,7 @@
           <t>Точно так</t>
         </is>
       </c>
-      <c r="C62" t="n">
+      <c r="C62" s="1" t="n">
         <v>0.250501002004008</v>
       </c>
     </row>
@@ -911,7 +935,7 @@
           <t>Важко відповісти</t>
         </is>
       </c>
-      <c r="C63" t="n">
+      <c r="C63" s="1" t="n">
         <v>0.2044088176352706</v>
       </c>
     </row>
@@ -921,7 +945,7 @@
           <t>Не хочу відповідати</t>
         </is>
       </c>
-      <c r="C64" t="n">
+      <c r="C64" s="1" t="n">
         <v>0.001002004008016032</v>
       </c>
     </row>
@@ -940,7 +964,7 @@
           <t>Точно ні</t>
         </is>
       </c>
-      <c r="C68" t="n">
+      <c r="C68" s="1" t="n">
         <v>0.01506024096385542</v>
       </c>
     </row>
@@ -950,7 +974,7 @@
           <t>Скоріше ні</t>
         </is>
       </c>
-      <c r="C69" t="n">
+      <c r="C69" s="1" t="n">
         <v>0.04518072289156626</v>
       </c>
     </row>
@@ -960,7 +984,7 @@
           <t>Скоріше так</t>
         </is>
       </c>
-      <c r="C70" t="n">
+      <c r="C70" s="1" t="n">
         <v>0.283132530120482</v>
       </c>
     </row>
@@ -970,7 +994,7 @@
           <t>Точно так</t>
         </is>
       </c>
-      <c r="C71" t="n">
+      <c r="C71" s="1" t="n">
         <v>0.5190763052208835</v>
       </c>
     </row>
@@ -980,7 +1004,7 @@
           <t>Важко відповісти</t>
         </is>
       </c>
-      <c r="C72" t="n">
+      <c r="C72" s="1" t="n">
         <v>0.1355421686746988</v>
       </c>
     </row>
@@ -990,7 +1014,7 @@
           <t>Не хочу відповідати</t>
         </is>
       </c>
-      <c r="C73" t="n">
+      <c r="C73" s="1" t="n">
         <v>0.002008032128514056</v>
       </c>
     </row>
@@ -1009,8 +1033,8 @@
           <t>Підписка на канали, пов'язані з Україною</t>
         </is>
       </c>
-      <c r="C77" t="n">
-        <v>0.535</v>
+      <c r="C77" s="1" t="n">
+        <v>0.5344655344655345</v>
       </c>
     </row>
     <row r="78">
@@ -1019,8 +1043,8 @@
           <t>Фотографування або публікація фотографій</t>
         </is>
       </c>
-      <c r="C78" t="n">
-        <v>0.518</v>
+      <c r="C78" s="1" t="n">
+        <v>0.5174825174825175</v>
       </c>
     </row>
     <row r="79">
@@ -1029,7 +1053,7 @@
           <t>Спілкування з людьми на підконтрольній Україні території (ПТУ)</t>
         </is>
       </c>
-      <c r="C79" t="n">
+      <c r="C79" s="1" t="n">
         <v>0.49</v>
       </c>
     </row>
@@ -1039,7 +1063,7 @@
           <t>Встановлення програм для забезпечення приватності (наприклад, VPN)</t>
         </is>
       </c>
-      <c r="C80" t="n">
+      <c r="C80" s="1" t="n">
         <v>0.379</v>
       </c>
     </row>
@@ -1049,7 +1073,7 @@
           <t>Використання Telegram</t>
         </is>
       </c>
-      <c r="C81" t="n">
+      <c r="C81" s="1" t="n">
         <v>0.376</v>
       </c>
     </row>
@@ -1059,7 +1083,7 @@
           <t>Наявність двох телефонів</t>
         </is>
       </c>
-      <c r="C82" t="n">
+      <c r="C82" s="1" t="n">
         <v>0.357</v>
       </c>
     </row>
@@ -1069,8 +1093,8 @@
           <t>Отримання грошових переказів з України</t>
         </is>
       </c>
-      <c r="C83" t="n">
-        <v>0.354</v>
+      <c r="C83" s="1" t="n">
+        <v>0.3546453546453546</v>
       </c>
     </row>
     <row r="84">
@@ -1079,10 +1103,8 @@
           <t>Інше</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>14.9%</t>
-        </is>
+      <c r="C84" s="1" t="n">
+        <v>0.1488511488511489</v>
       </c>
     </row>
     <row r="85">
@@ -1091,7 +1113,7 @@
           <t>Важко відповісти</t>
         </is>
       </c>
-      <c r="C85" t="n">
+      <c r="C85" s="1" t="n">
         <v>0.212</v>
       </c>
     </row>
@@ -1101,7 +1123,7 @@
           <t>Не хочу відповідати</t>
         </is>
       </c>
-      <c r="C86" t="n">
+      <c r="C86" s="1" t="n">
         <v>0.004</v>
       </c>
     </row>
@@ -1120,7 +1142,7 @@
           <t>Допомога людям у безпечній евакуації з ТОТ (тимчасово окупованих територій) на підконтрольну Україні територію (ПТУ)</t>
         </is>
       </c>
-      <c r="C90" t="n">
+      <c r="C90" s="1" t="n">
         <v>0.465</v>
       </c>
     </row>
@@ -1130,7 +1152,7 @@
           <t>Постачання медикаментів цивільним особам</t>
         </is>
       </c>
-      <c r="C91" t="n">
+      <c r="C91" s="1" t="n">
         <v>0.428</v>
       </c>
     </row>
@@ -1140,7 +1162,7 @@
           <t>Надання товарів першої необхідності, яких бракує (наприклад, таблетки для очищення води, засоби гігієни, дитячі суміші)</t>
         </is>
       </c>
-      <c r="C92" t="n">
+      <c r="C92" s="1" t="n">
         <v>0.415</v>
       </c>
     </row>
@@ -1150,7 +1172,7 @@
           <t>Надання юридичної підтримки учасникам громадянського спротиву, ув'язненим російською владою</t>
         </is>
       </c>
-      <c r="C93" t="n">
+      <c r="C93" s="1" t="n">
         <v>0.359</v>
       </c>
     </row>
@@ -1160,7 +1182,7 @@
           <t>Надання безпечних засобів зв'язку для відстеження переміщень російських військ</t>
         </is>
       </c>
-      <c r="C94" t="n">
+      <c r="C94" s="1" t="n">
         <v>0.316</v>
       </c>
     </row>
@@ -1170,7 +1192,7 @@
           <t>поширення проукраїнського чи антиокупаційного контенту в Telegram, TikTok чи на інших платформах</t>
         </is>
       </c>
-      <c r="C95" t="n">
+      <c r="C95" s="1" t="n">
         <v>0.295</v>
       </c>
     </row>
@@ -1180,7 +1202,7 @@
           <t>Публікація або розповсюдження публічних списків колаборантів</t>
         </is>
       </c>
-      <c r="C96" t="n">
+      <c r="C96" s="1" t="n">
         <v>0.292</v>
       </c>
     </row>
@@ -1190,7 +1212,7 @@
           <t>Організація пасивного спротиву (наприклад, бойкот організованих Росією заходів, відмова від російських паспортів)</t>
         </is>
       </c>
-      <c r="C97" t="n">
+      <c r="C97" s="1" t="n">
         <v>0.26</v>
       </c>
     </row>
@@ -1200,7 +1222,7 @@
           <t>Фотографування з українською символікою (стрічки, плакати) та публікація фотографій онлайн</t>
         </is>
       </c>
-      <c r="C98" t="n">
+      <c r="C98" s="1" t="n">
         <v>0.255</v>
       </c>
     </row>
@@ -1210,7 +1232,7 @@
           <t>Підтримка місцевої кібер-обізнаності (наприклад, проведення базових тренінгів з цифрової безпеки офлайн)</t>
         </is>
       </c>
-      <c r="C99" t="n">
+      <c r="C99" s="1" t="n">
         <v>0.231</v>
       </c>
     </row>
@@ -1220,10 +1242,8 @@
           <t>Інше</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>8.8%</t>
-        </is>
+      <c r="C100" s="1" t="n">
+        <v>0.08791208791208792</v>
       </c>
     </row>
     <row r="101">
@@ -1232,8 +1252,8 @@
           <t>Важко відповісти</t>
         </is>
       </c>
-      <c r="C101" t="n">
-        <v>0.245</v>
+      <c r="C101" s="1" t="n">
+        <v>0.2457542457542458</v>
       </c>
     </row>
     <row r="102">
@@ -1242,7 +1262,7 @@
           <t>Не хочу відповідати</t>
         </is>
       </c>
-      <c r="C102" t="n">
+      <c r="C102" s="1" t="n">
         <v>0.018</v>
       </c>
     </row>
@@ -1270,7 +1290,7 @@
           <t>18–24</t>
         </is>
       </c>
-      <c r="C109" t="n">
+      <c r="C109" s="1" t="n">
         <v>0.04095904095904096</v>
       </c>
     </row>
@@ -1280,7 +1300,7 @@
           <t>25–34</t>
         </is>
       </c>
-      <c r="C110" t="n">
+      <c r="C110" s="1" t="n">
         <v>0.1398601398601399</v>
       </c>
     </row>
@@ -1290,7 +1310,7 @@
           <t>35–49</t>
         </is>
       </c>
-      <c r="C111" t="n">
+      <c r="C111" s="1" t="n">
         <v>0.3196803196803197</v>
       </c>
     </row>
@@ -1300,7 +1320,7 @@
           <t>50–59</t>
         </is>
       </c>
-      <c r="C112" t="n">
+      <c r="C112" s="1" t="n">
         <v>0.2147852147852148</v>
       </c>
     </row>
@@ -1310,7 +1330,7 @@
           <t>60+</t>
         </is>
       </c>
-      <c r="C113" t="n">
+      <c r="C113" s="1" t="n">
         <v>0.2847152847152847</v>
       </c>
     </row>
@@ -1329,7 +1349,7 @@
           <t>Чоловіча</t>
         </is>
       </c>
-      <c r="C117" t="n">
+      <c r="C117" s="1" t="n">
         <v>0.3606393606393606</v>
       </c>
     </row>
@@ -1339,277 +1359,18 @@
           <t>Жіноча</t>
         </is>
       </c>
-      <c r="C118" t="n">
+      <c r="C118" s="1" t="n">
         <v>0.6393606393606394</v>
       </c>
     </row>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181">
-      <c r="B181" t="n">
-        <v>0.2324844266</v>
-      </c>
-    </row>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Виправлено у жовтні 2026 р. (Q7, Q8, Q11, Q12): див. аркуш «Виправлення (Corrections)».</t>
+        </is>
+      </c>
+    </row>
+    <row r="181"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1621,10 +1382,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z305"/>
+  <dimension ref="B2:C105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -2667,206 +2427,6 @@
         </is>
       </c>
     </row>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2878,10 +2438,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y258"/>
+  <dimension ref="B2:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -3454,206 +3013,336 @@
         </is>
       </c>
     </row>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Виправлення, жовтень 2026 / Corrections, October 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Питання / Question</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Відповідь / Answer</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Було / Originally published</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Стало / Corrected</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Причина / Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Q8 Most of the population remaining in the occupied territories is satisfied with the Russian authorities</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Definitely no</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>3.6%</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>26.2%</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Distribution copied from Q9 in error</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Rather no</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>32.4%</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Distribution copied from Q9 in error</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Rather yes</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>36.5%</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>19.8%</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Distribution copied from Q9 in error</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Definitely yes</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>25.1%</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Distribution copied from Q9 in error</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Q7 Do you keep in touch with acquaintances in the occupied territories?</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Hard to say</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0.5%</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>0.8%</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Transposed with "prefer not to answer"</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Prefer not to answer</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0.8%</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>0.5%</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Transposed with "hard to say"</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Q11 Behaviours that may create a risk of violence</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Subscribing to Ukraine-related channels</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>53.5%</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>53.4%</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Rounding (535 of 1,001)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Taking or publishing photos</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>51.8%</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>51.7%</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Rounding (518 of 1,001)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Receiving money transfers from Ukraine</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>35.4%</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>35.5%</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Rounding (355 of 1,001)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Q12 Non-violent actions worth the risk</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Hard to say</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>24.5%</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>24.6%</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Rounding (246 of 1,001)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Усі значення перевірено за масивом відповідей 2025 р. / All values were checked against the 2025 respondent-level file.</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Хвиля 2026 р. / 2026 wave: https://totinsights.org/idp-survey-2026.html</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>